<commit_message>
Adopt canonical PET/PEESE selection rule
</commit_message>
<xml_diff>
--- a/4_tables/2_meta_analysis/meta_housing_ma_ground.xlsx
+++ b/4_tables/2_meta_analysis/meta_housing_ma_ground.xlsx
@@ -412,12 +412,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.910 [0.836, 0.989]</t>
+          <t>0.957 [0.886, 1.033]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
     </row>
@@ -476,12 +476,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.954 [0.928, 0.980]</t>
+          <t>0.984 [0.963, 1.005]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -849,90 +849,125 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>pet_p_value</t>
+          <t>bc_estimate</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>bc_std_error</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>bc_statistic</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>bc_p_value</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>bc_alpha</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>bc_direction_used</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>selector_note</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>pet_term_p_value_diag</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>pet_status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>peese_status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>fit_status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>fit_note</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>pet_term</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>model_formula</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>estimate_rr</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>std_error</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>conf_low</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>conf_high</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>conf_low_rr</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>conf_high_rr</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>pet_term_estimate</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>pet_term_p_value</t>
         </is>
@@ -967,74 +1002,94 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="J2">
+        <v>-0.0441289342241922</v>
+      </c>
+      <c r="K2">
+        <v>0.039294877575553</v>
+      </c>
+      <c r="L2">
+        <v>-1.123020020595424</v>
+      </c>
+      <c r="M2">
+        <v>0.2614289916605104</v>
+      </c>
+      <c r="N2">
+        <v>0.1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="Q2">
         <v>8.801475483338173E-05</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>prratio_ln_v</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>prratio_ln ~ 1 + prratio_ln_v | 0</t>
-        </is>
-      </c>
-      <c r="Q2">
-        <v>-0.09483426427679595</v>
-      </c>
-      <c r="R2">
-        <v>0.9095236625393556</v>
-      </c>
-      <c r="S2">
-        <v>0.04271964348708504</v>
-      </c>
-      <c r="T2">
-        <v>-2.219921716000887</v>
-      </c>
-      <c r="U2">
-        <v>0.02885430705018921</v>
-      </c>
-      <c r="V2">
-        <v>-0.1785632269438737</v>
-      </c>
-      <c r="W2">
-        <v>-0.0111053016097182</v>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>prratio_ln_se</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>prratio_ln ~ 1 + prratio_ln_se | 0</t>
+        </is>
       </c>
       <c r="X2">
-        <v>0.8364711676898278</v>
+        <v>-0.0441289342241922</v>
       </c>
       <c r="Y2">
-        <v>0.9889561346192752</v>
+        <v>0.956830581310828</v>
       </c>
       <c r="Z2">
-        <v>-6.964456385847269</v>
+        <v>0.03929487743047507</v>
       </c>
       <c r="AA2">
-        <v>0.009633536968474372</v>
+        <v>-1.12302002474165</v>
+      </c>
+      <c r="AB2">
+        <v>0.2643197630713425</v>
+      </c>
+      <c r="AC2">
+        <v>-0.1211454787648392</v>
+      </c>
+      <c r="AD2">
+        <v>0.03288761031645475</v>
+      </c>
+      <c r="AE2">
+        <v>0.8859050698424167</v>
+      </c>
+      <c r="AF2">
+        <v>1.033434385350644</v>
+      </c>
+      <c r="AG2">
+        <v>-2.171136979968024</v>
+      </c>
+      <c r="AH2">
+        <v>8.801475483338173E-05</v>
       </c>
     </row>
     <row r="3">
@@ -1075,64 +1130,84 @@
         </is>
       </c>
       <c r="J3">
+        <v>0.01886571046568258</v>
+      </c>
+      <c r="K3">
+        <v>0.04777190213453326</v>
+      </c>
+      <c r="L3">
+        <v>0.3949122731716596</v>
+      </c>
+      <c r="M3">
+        <v>0.6929076319857237</v>
+      </c>
+      <c r="N3">
+        <v>0.1</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="Q3">
         <v>0.6896331316971431</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>prratio_ln_se</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>prratio_ln ~ 1 + prratio_ln_se | 0</t>
         </is>
       </c>
-      <c r="Q3">
+      <c r="X3">
         <v>0.01886571046568258</v>
       </c>
-      <c r="R3">
+      <c r="Y3">
         <v>1.019044792377816</v>
       </c>
-      <c r="S3">
+      <c r="Z3">
         <v>0.04777190240922339</v>
       </c>
-      <c r="T3">
+      <c r="AA3">
         <v>0.3949122709009</v>
       </c>
-      <c r="U3">
+      <c r="AB3">
         <v>0.6960102049424469</v>
       </c>
-      <c r="V3">
+      <c r="AC3">
         <v>-0.07476549772935748</v>
       </c>
-      <c r="W3">
+      <c r="AD3">
         <v>0.1124969186607226</v>
       </c>
-      <c r="X3">
+      <c r="AE3">
         <v>0.9279610697935819</v>
       </c>
-      <c r="Y3">
+      <c r="AF3">
         <v>1.119068808676794</v>
       </c>
-      <c r="Z3">
+      <c r="AG3">
         <v>0.2119180839801686</v>
       </c>
-      <c r="AA3">
+      <c r="AH3">
         <v>0.6896331316971431</v>
       </c>
     </row>
@@ -1165,74 +1240,94 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>peese</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="J4">
+        <v>-0.01623317719789098</v>
+      </c>
+      <c r="K4">
+        <v>0.01085249306634288</v>
+      </c>
+      <c r="L4">
+        <v>-1.495801664986579</v>
+      </c>
+      <c r="M4">
+        <v>0.1347053473598521</v>
+      </c>
+      <c r="N4">
+        <v>0.1</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="Q4">
         <v>0.00152539740558465</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>prratio_ln_v</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>prratio_ln ~ 1 + prratio_ln_v | 0</t>
-        </is>
-      </c>
-      <c r="Q4">
-        <v>-0.04736005941814025</v>
-      </c>
-      <c r="R4">
-        <v>0.9537439312749914</v>
-      </c>
-      <c r="S4">
-        <v>0.01394608033199637</v>
-      </c>
-      <c r="T4">
-        <v>-3.395940528858311</v>
-      </c>
-      <c r="U4">
-        <v>0.004779457142527119</v>
-      </c>
-      <c r="V4">
-        <v>-0.07469387459435553</v>
-      </c>
-      <c r="W4">
-        <v>-0.02002624424192496</v>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>prratio_ln_se</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>prratio_ln ~ 1 + prratio_ln_se | 0</t>
+        </is>
       </c>
       <c r="X4">
-        <v>0.9280275356547786</v>
+        <v>-0.01623317719789098</v>
       </c>
       <c r="Y4">
-        <v>0.9801729490731965</v>
+        <v>0.9838978707566386</v>
       </c>
       <c r="Z4">
-        <v>-9.791893465386963</v>
+        <v>0.01085249309360055</v>
       </c>
       <c r="AA4">
-        <v>0.02225205193640684</v>
+        <v>-1.495801661229649</v>
+      </c>
+      <c r="AB4">
+        <v>0.1585823524778318</v>
+      </c>
+      <c r="AC4">
+        <v>-0.03750367280381772</v>
+      </c>
+      <c r="AD4">
+        <v>0.005037318408035753</v>
+      </c>
+      <c r="AE4">
+        <v>0.9631908801031837</v>
+      </c>
+      <c r="AF4">
+        <v>1.005050027026566</v>
+      </c>
+      <c r="AG4">
+        <v>-2.105870116707555</v>
+      </c>
+      <c r="AH4">
+        <v>0.00152539740558465</v>
       </c>
     </row>
     <row r="5">
@@ -1273,64 +1368,84 @@
         </is>
       </c>
       <c r="J5">
+        <v>-0.01650615869253858</v>
+      </c>
+      <c r="K5">
+        <v>0.02676725555339267</v>
+      </c>
+      <c r="L5">
+        <v>-0.6166548774346226</v>
+      </c>
+      <c r="M5">
+        <v>0.537462389575474</v>
+      </c>
+      <c r="N5">
+        <v>0.1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="Q5">
         <v>0.2130269863307577</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>prratio_ln_se</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>prratio_ln ~ 1 + prratio_ln_se | 0</t>
         </is>
       </c>
-      <c r="Q5">
+      <c r="X5">
         <v>-0.01650615869253858</v>
       </c>
-      <c r="R5">
+      <c r="Y5">
         <v>0.983629321501455</v>
       </c>
-      <c r="S5">
+      <c r="Z5">
         <v>0.0267672554654336</v>
       </c>
-      <c r="T5">
+      <c r="AA5">
         <v>-0.6166548794609935</v>
       </c>
-      <c r="U5">
+      <c r="AB5">
         <v>0.5456327536525746</v>
       </c>
-      <c r="V5">
+      <c r="AC5">
         <v>-0.06896901536977135</v>
       </c>
-      <c r="W5">
+      <c r="AD5">
         <v>0.03595669798469419</v>
       </c>
-      <c r="X5">
+      <c r="AE5">
         <v>0.9333555993082903</v>
       </c>
-      <c r="Y5">
+      <c r="AF5">
         <v>1.036610958175476</v>
       </c>
-      <c r="Z5">
+      <c r="AG5">
         <v>-0.4058176217004146</v>
       </c>
-      <c r="AA5">
+      <c r="AH5">
         <v>0.2130269863307577</v>
       </c>
     </row>
@@ -1372,64 +1487,84 @@
         </is>
       </c>
       <c r="J6">
+        <v>-0.1514253255935879</v>
+      </c>
+      <c r="K6">
+        <v>0.1500586848950155</v>
+      </c>
+      <c r="L6">
+        <v>-1.009107374888221</v>
+      </c>
+      <c r="M6">
+        <v>0.3129231414725175</v>
+      </c>
+      <c r="N6">
+        <v>0.1</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="Q6">
         <v>0.3518414027608091</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>prratio_ln_se</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>prratio_ln ~ 1 + prratio_ln_se | 0</t>
         </is>
       </c>
-      <c r="Q6">
+      <c r="X6">
         <v>-0.1514253255935879</v>
       </c>
-      <c r="R6">
+      <c r="Y6">
         <v>0.8594820611893771</v>
       </c>
-      <c r="S6">
+      <c r="Z6">
         <v>0.1500586842514219</v>
       </c>
-      <c r="T6">
+      <c r="AA6">
         <v>-1.009107379216228</v>
       </c>
-      <c r="U6">
+      <c r="AB6">
         <v>0.3238937376980864</v>
       </c>
-      <c r="V6">
+      <c r="AC6">
         <v>-0.4455349422938426</v>
       </c>
-      <c r="W6">
+      <c r="AD6">
         <v>0.1426842911066667</v>
       </c>
-      <c r="X6">
+      <c r="AE6">
         <v>0.6404815636979818</v>
       </c>
-      <c r="Y6">
+      <c r="AF6">
         <v>1.15336561639841</v>
       </c>
-      <c r="Z6">
+      <c r="AG6">
         <v>-1.66112279063935</v>
       </c>
-      <c r="AA6">
+      <c r="AH6">
         <v>0.3518414027608091</v>
       </c>
     </row>
@@ -1440,7 +1575,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1481,22 +1616,57 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>pet_p_value</t>
+          <t>pet_status</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>pet_status</t>
+          <t>peese_status</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>peese_status</t>
+          <t>selected_model</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>selected_model</t>
+          <t>bc_estimate</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>bc_std_error</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>bc_statistic</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>bc_p_value</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>bc_alpha</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>bc_direction_used</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>selector_note</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>pet_term_p_value_diag</t>
         </is>
       </c>
     </row>
@@ -1527,23 +1697,43 @@
       <c r="G2">
         <v>94</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="K2">
+        <v>-0.0441289342241922</v>
+      </c>
+      <c r="L2">
+        <v>0.039294877575553</v>
+      </c>
+      <c r="M2">
+        <v>-1.123020020595424</v>
+      </c>
+      <c r="N2">
+        <v>0.2614289916605104</v>
+      </c>
+      <c r="O2">
+        <v>0.1</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="R2">
         <v>8.801475483338173E-05</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>peese</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -1573,23 +1763,43 @@
       <c r="G3">
         <v>28</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="K3">
+        <v>0.01886571046568258</v>
+      </c>
+      <c r="L3">
+        <v>0.04777190213453326</v>
+      </c>
+      <c r="M3">
+        <v>0.3949122731716596</v>
+      </c>
+      <c r="N3">
+        <v>0.6929076319857237</v>
+      </c>
+      <c r="O3">
+        <v>0.1</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="R3">
         <v>0.6896331316971431</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>pet</t>
-        </is>
       </c>
     </row>
     <row r="4">
@@ -1619,23 +1829,43 @@
       <c r="G4">
         <v>14</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="K4">
+        <v>-0.01623317719789098</v>
+      </c>
+      <c r="L4">
+        <v>0.01085249306634288</v>
+      </c>
+      <c r="M4">
+        <v>-1.495801664986579</v>
+      </c>
+      <c r="N4">
+        <v>0.1347053473598521</v>
+      </c>
+      <c r="O4">
+        <v>0.1</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="R4">
         <v>0.00152539740558465</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>peese</t>
-        </is>
       </c>
     </row>
     <row r="5">
@@ -1665,23 +1895,43 @@
       <c r="G5">
         <v>18</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="K5">
+        <v>-0.01650615869253858</v>
+      </c>
+      <c r="L5">
+        <v>0.02676725555339267</v>
+      </c>
+      <c r="M5">
+        <v>-0.6166548774346226</v>
+      </c>
+      <c r="N5">
+        <v>0.537462389575474</v>
+      </c>
+      <c r="O5">
+        <v>0.1</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="R5">
         <v>0.2130269863307577</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>pet</t>
-        </is>
       </c>
     </row>
     <row r="6">
@@ -1711,23 +1961,43 @@
       <c r="G6">
         <v>23</v>
       </c>
-      <c r="H6">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="K6">
+        <v>-0.1514253255935879</v>
+      </c>
+      <c r="L6">
+        <v>0.1500586848950155</v>
+      </c>
+      <c r="M6">
+        <v>-1.009107374888221</v>
+      </c>
+      <c r="N6">
+        <v>0.3129231414725175</v>
+      </c>
+      <c r="O6">
+        <v>0.1</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="R6">
         <v>0.3518414027608091</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>pet</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>